<commit_message>
redesign canonical Excel templates and add complex example
</commit_message>
<xml_diff>
--- a/ct/tests/fixtures/repository_cutover/workspace/excel/Item.xlsx
+++ b/ct/tests/fixtures/repository_cutover/workspace/excel/Item.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,15 +26,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
+      <name val="Aptos"/>
+      <color rgb="00334155"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -47,30 +40,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C9A227"/>
-        <bgColor rgb="00C9A227"/>
+        <fgColor rgb="0092400E"/>
+        <bgColor rgb="0092400E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00E2E8F0"/>
+        <bgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B4332"/>
-        <bgColor rgb="001B4332"/>
+        <fgColor rgb="00166534"/>
+        <bgColor rgb="00166534"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0040916C"/>
-        <bgColor rgb="0040916C"/>
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -85,25 +78,72 @@
       <bottom style="thin"/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
       <left style="thin"/>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="00334155"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="00334155"/>
+      </bottom>
     </border>
     <border>
       <left style="thin"/>
       <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="double">
+        <color rgb="00334155"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
+      <bottom style="double">
+        <color rgb="00334155"/>
+      </bottom>
     </border>
     <border>
       <left/>
@@ -130,59 +170,88 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00EDF7EE"/>
-          <bgColor rgb="00EDF7EE"/>
+          <fgColor rgb="00F8FAFC"/>
+          <bgColor rgb="00F8FAFC"/>
         </patternFill>
       </fill>
-      <border>
-        <left style="thin">
-          <color rgb="00CCCCCC"/>
-        </left>
-        <right style="thin">
-          <color rgb="00CCCCCC"/>
-        </right>
-      </border>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="00581C87"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
-          <bgColor rgb="00FFFFFF"/>
+          <fgColor rgb="00F3E8FF"/>
         </patternFill>
       </fill>
-      <border>
-        <left style="thin">
-          <color rgb="00CCCCCC"/>
-        </left>
-        <right style="thin">
-          <color rgb="00CCCCCC"/>
-        </right>
-      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00155E75"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00ECFEFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00475569"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F1F5F9"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -255,6 +324,24 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ct</author>
+  </authors>
+  <commentList>
+    <comment ref="D2" authorId="0" shapeId="0">
+      <text>
+        <t>类型：ItemRarity；稀有度
+common: 普通
+rare: 稀有
+epic: 史诗</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -560,189 +647,164 @@
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>道具唯一ID，禁止修改</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>道具名称（多语言）</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>售价（金币），0=不可出售</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>稀有度</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>道具类型，关联 ItemType.Id</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>掉落数量下限</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>标签列表，使用 [1,2,3] 文法</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>是否启用（仅服务端）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Id
 int32</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Name
-string[i18n]</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+string</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Price
 float</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Rarity
-enum[common,rare,epic]</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+ItemRarity</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>ItemTypeId
-int32[ref:ItemType.Id]</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
+int32</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>DropRange
-Droprange</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="2" t="inlineStr">
+ItemDropRange</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="n"/>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Tags
-array&lt;int32&gt;</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
+vector&lt;int32&gt;</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>IsActive
 bool</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="7" t="n"/>
-      <c r="B2" s="7" t="n"/>
-      <c r="C2" s="7" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>掉落数量下限</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>掉落数量上限</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="n"/>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="10" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Min
-int32</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+ItemDropRange</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Max
-int32</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>道具唯一ID，禁止修改</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>道具名称（多语言）</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>售价（金币），0=不可出售</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>稀有度</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>道具类型，关联 ItemType.Id</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>掉落数量下限</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>掉落数量上限</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>标签列表，逗号分隔</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>是否启用（仅服务端）</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>药水</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>common</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>101,102</t>
-        </is>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
+ItemDropRange</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>铁剑</t>
+          <t>药水</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>100</v>
+        <v>10.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>[101,102]</t>
         </is>
       </c>
       <c r="I5" t="b">
@@ -751,98 +813,194 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>魔法石</t>
+          <t>铁剑</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>epic</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>301,302,303</t>
+          <t>[201]</t>
         </is>
       </c>
       <c r="I6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>魔法石</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[301,302,303]</t>
+        </is>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>面包</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C8" t="n">
         <v>5</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G8" t="n">
         <v>10</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="I7" t="b">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[101]</t>
+        </is>
+      </c>
+      <c r="I8" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="I1:I2"/>
+  <mergeCells count="2">
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:I1000">
+  <conditionalFormatting sqref="A5:A1048576">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>MOD(ROW(),2)=1</formula>
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="D4:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <conditionalFormatting sqref="B5:B1048576">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:C1048576">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D1048576">
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>D5&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5:E1048576">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>E5&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F1048576">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G1048576">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H1048576">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>AND($A5&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I1048576">
+    <cfRule type="expression" priority="9" dxfId="3">
+      <formula>I5=TRUE</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="4">
+      <formula>I5=FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="8">
+    <dataValidation sqref="A5:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation sqref="C5:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
+      <formula1>-1E+307</formula1>
+      <formula2>1E+307</formula2>
+    </dataValidation>
+    <dataValidation sqref="D5:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"common,rare,epic"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="引用" prompt="目标：ItemType.Id；最终以 canonical 校验为准" type="custom">
+      <formula1>TRUE</formula1>
+    </dataValidation>
+    <dataValidation sqref="F5:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation sqref="G5:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation sqref="H5:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+      <formula1>-2147483648</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation sqref="I5:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>